<commit_message>
[ENH] Updated protocol and instructions
</commit_message>
<xml_diff>
--- a/src/instructions/[ES]WELCOME_SCREEN.xlsx
+++ b/src/instructions/[ES]WELCOME_SCREEN.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\akoun\Desktop\Biocruces\begibraintool\src\instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CFD19D6-91F9-4956-8B53-728D8FC8E6AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE2C6D91-8815-4B3E-A241-4E3B630BE849}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8205" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -117,9 +117,9 @@
   </si>
   <si>
     <t>¡Bienvenido/a! Gracias por participar en este estudio.
-A continuación realizarás una serie de pruebas visuales. Durante las pruebas, solo tienes que seguir las instrucciones que aparecerán en pantalla.
+Durante esta visita realizarás una serie de pruebas visuales. Antes de cada prueba habra una pantalla como esta en la que se explica lo que tienes que hacer.
 No hay respuestas buenas ni malas. Si en algún momento te equivocas, no pasa nada.
-Pulsa el botón central para comenzar.</t>
+Pulsa el botón central para comenzar con las instrucciones de la primera prueba.</t>
   </si>
 </sst>
 </file>
@@ -570,6 +570,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B9F5CAB0486A994CA2C3B13E059EF2AE" ma:contentTypeVersion="0" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="8645ec4a60d0c8c7009d2d6675847a91">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="636d7205651659ec4fcda0bcbde9384b">
     <xsd:element name="properties">
@@ -683,22 +698,30 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3744155D-8FAB-4E67-B5E0-C7FDBFB3715D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3725960-8A89-4E70-9C40-340E0EDB6403}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFF1C174-6AC6-4774-A736-3226A12360E4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -712,27 +735,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3725960-8A89-4E70-9C40-340E0EDB6403}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3744155D-8FAB-4E67-B5E0-C7FDBFB3715D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>